<commit_message>
Update hardware case and PCB assets
</commit_message>
<xml_diff>
--- a/hardware/DuploTrainController NG/5 Buttons an ADC.xlsx
+++ b/hardware/DuploTrainController NG/5 Buttons an ADC.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ralf/Desktop/Projekte von Workbench/20_Duplo Train Controller NG/ControllerHW/DuploTrainController NG/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/SSD1000/2_Workbench/2_HW_Projekte/4_Realisierte_Projekte/20_Duplo Train Controller NG/DuploTrain-NG/hardware/DuploTrainController NG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E8145A7-D63D-E84F-9C49-DD355DA80156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78900CBA-AB6F-514C-8BB2-4656FABF8632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" xr2:uid="{3208A821-9F98-A04C-982F-D10FE78BA69E}"/>
+    <workbookView xWindow="-30620" yWindow="1340" windowWidth="28800" windowHeight="16260" xr2:uid="{3208A821-9F98-A04C-982F-D10FE78BA69E}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
   <si>
     <t>R1</t>
   </si>
@@ -131,6 +131,18 @@
   </si>
   <si>
     <t>R E12 in k</t>
+  </si>
+  <si>
+    <t>ADC Wert</t>
+  </si>
+  <si>
+    <t>Sound</t>
+  </si>
+  <si>
+    <t>Light</t>
+  </si>
+  <si>
+    <t>Button</t>
   </si>
 </sst>
 </file>
@@ -139,7 +151,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="171" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -176,11 +188,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -495,313 +508,366 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89797360-B5FE-4F4C-8CDE-BD5A4372B6AA}">
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:S13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="5" max="5" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="13" max="13" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15" customWidth="1"/>
+    <col min="14" max="14" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>1</v>
       </c>
-      <c r="B1">
+      <c r="C1">
         <v>2.2000000000000002</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>10</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>14</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>15</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>31</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>16</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="Q1" t="s">
+        <v>32</v>
+      </c>
+      <c r="S1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>21</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>0</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>22</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B3">
+      <c r="C3">
         <v>0.15</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>0</v>
       </c>
-      <c r="E3" s="1">
-        <f>B3/(1-B3)*$B$1</f>
+      <c r="F3" s="1">
+        <f t="shared" ref="F3:F8" si="0">C3/(1-C3)*$C$1</f>
         <v>0.38823529411764712</v>
       </c>
-      <c r="F3" s="1">
-        <f>E3</f>
+      <c r="G3" s="1">
+        <f>F3</f>
         <v>0.38823529411764712</v>
       </c>
-      <c r="G3">
-        <f>B3*3.3</f>
+      <c r="H3">
+        <f>C3*3.3</f>
         <v>0.49499999999999994</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>23</v>
       </c>
-      <c r="K3">
-        <v>0.39</v>
-      </c>
-      <c r="M3" s="3">
-        <f>$C$12*K3/($B$1+K3)</f>
-        <v>0.49691119691119684</v>
+      <c r="L3">
+        <v>0.43</v>
       </c>
       <c r="N3" s="3">
-        <f>M3</f>
-        <v>0.49691119691119684</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+        <f>$D$12*L3/($C$1+L3)</f>
+        <v>0.53954372623574132</v>
+      </c>
+      <c r="O3" s="3">
+        <f>N3</f>
+        <v>0.53954372623574132</v>
+      </c>
+      <c r="Q3" s="4">
+        <f>N3/$N$9*4096</f>
+        <v>669.68821292775658</v>
+      </c>
+      <c r="S3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4">
+      <c r="C4">
         <v>0.3</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="1">
-        <f>B4/(1-B4)*$B$1</f>
+      <c r="F4" s="1">
+        <f t="shared" si="0"/>
         <v>0.94285714285714295</v>
       </c>
-      <c r="F4" s="1">
-        <f>E4-F3</f>
+      <c r="G4" s="1">
+        <f>F4-G3</f>
         <v>0.55462184873949583</v>
       </c>
-      <c r="G4">
-        <f t="shared" ref="G4:G7" si="0">B4*3.3</f>
+      <c r="H4">
+        <f t="shared" ref="H4:H7" si="1">C4*3.3</f>
         <v>0.98999999999999988</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>24</v>
       </c>
-      <c r="K4">
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="M4" s="3">
-        <f>$C$12*(K4+K3)/($B$1+K4+K3)</f>
-        <v>0.99523809523809514</v>
+      <c r="L4">
+        <v>0.62</v>
       </c>
       <c r="N4" s="3">
-        <f>M4-M3</f>
-        <v>0.4983268983268983</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+        <f>$D$12*(L4+L3)/($C$1+L4+L3)</f>
+        <v>1.066153846153846</v>
+      </c>
+      <c r="O4" s="3">
+        <f>N4-N3</f>
+        <v>0.52661011991810469</v>
+      </c>
+      <c r="Q4" s="4">
+        <f t="shared" ref="Q4:Q9" si="2">N4/$N$9*4096</f>
+        <v>1323.3230769230768</v>
+      </c>
+      <c r="S4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="B5">
+      <c r="C5">
         <v>0.45</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="1">
-        <f>B5/(1-B5)*$B$1</f>
+      <c r="F5" s="1">
+        <f t="shared" si="0"/>
         <v>1.8</v>
       </c>
-      <c r="F5" s="1">
-        <f>E5-E4</f>
+      <c r="G5" s="1">
+        <f>F5-F4</f>
         <v>0.8571428571428571</v>
       </c>
-      <c r="G5">
-        <f t="shared" si="0"/>
+      <c r="H5">
+        <f t="shared" si="1"/>
         <v>1.4849999999999999</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>25</v>
       </c>
-      <c r="K5">
-        <v>0.82</v>
-      </c>
-      <c r="M5" s="3">
-        <f>$C$12*(K5+K4+K3)/($B$1+K5+K4+K3)</f>
-        <v>1.4712846347607051</v>
+      <c r="L5">
+        <v>0.91</v>
       </c>
       <c r="N5" s="3">
-        <f t="shared" ref="N5:N9" si="1">M5-M4</f>
-        <v>0.47604653952261</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+        <f>$D$12*(L5+L4+L3)/($C$1+L5+L4+L3)</f>
+        <v>1.5548076923076923</v>
+      </c>
+      <c r="O5" s="3">
+        <f t="shared" ref="O5:O9" si="3">N5-N4</f>
+        <v>0.48865384615384633</v>
+      </c>
+      <c r="Q5" s="4">
+        <f t="shared" si="2"/>
+        <v>1929.846153846154</v>
+      </c>
+      <c r="S5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6">
+      <c r="C6">
         <v>0.6</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="1">
-        <f>B6/(1-B6)*$B$1</f>
+      <c r="F6" s="1">
+        <f t="shared" si="0"/>
         <v>3.3</v>
       </c>
-      <c r="F6" s="1">
-        <f>E6-E5</f>
+      <c r="G6" s="1">
+        <f>F6-F5</f>
         <v>1.4999999999999998</v>
       </c>
-      <c r="G6">
-        <f t="shared" si="0"/>
+      <c r="H6">
+        <f t="shared" si="1"/>
         <v>1.9799999999999998</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>26</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>1.5</v>
       </c>
-      <c r="M6" s="3">
-        <f>$C$12*(K6+K5+K4+K3)/($B$1+K6+K5+K4+K3)</f>
-        <v>1.9727605118829981</v>
-      </c>
       <c r="N6" s="3">
-        <f t="shared" si="1"/>
-        <v>0.50147587712229291</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+        <f>$D$12*(L6+L5+L4+L3)/($C$1+L6+L5+L4+L3)</f>
+        <v>2.0173144876325089</v>
+      </c>
+      <c r="O6" s="3">
+        <f t="shared" si="3"/>
+        <v>0.46250679532481653</v>
+      </c>
+      <c r="Q6" s="4">
+        <f t="shared" si="2"/>
+        <v>2503.9151943462898</v>
+      </c>
+      <c r="S6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>9</v>
       </c>
-      <c r="B7">
+      <c r="C7">
         <v>0.75</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="1">
-        <f>B7/(1-B7)*$B$1</f>
+      <c r="F7" s="1">
+        <f t="shared" si="0"/>
         <v>6.6000000000000005</v>
       </c>
-      <c r="F7" s="1">
-        <f>E7-E6</f>
+      <c r="G7" s="1">
+        <f>F7-F6</f>
         <v>3.3000000000000007</v>
       </c>
-      <c r="G7">
-        <f t="shared" si="0"/>
+      <c r="H7">
+        <f t="shared" si="1"/>
         <v>2.4749999999999996</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>27</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>3.3</v>
       </c>
-      <c r="M7" s="3">
-        <f>$C$12*(K7+K6+K5+K4+K3)/($B$1+K7+K6+K5+K4+K3)</f>
-        <v>2.4721778791334086</v>
-      </c>
       <c r="N7" s="3">
-        <f t="shared" si="1"/>
-        <v>0.49941736725041053</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+        <f>$D$12*(L7+L6+L5+L4+L3)/($C$1+L7+L6+L5+L4+L3)</f>
+        <v>2.4897321428571431</v>
+      </c>
+      <c r="O7" s="3">
+        <f t="shared" si="3"/>
+        <v>0.47241765522463419</v>
+      </c>
+      <c r="Q7" s="4">
+        <f t="shared" si="2"/>
+        <v>3090.2857142857147</v>
+      </c>
+      <c r="S7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>18</v>
       </c>
-      <c r="B8">
+      <c r="C8">
         <v>0.9</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="1">
-        <f>B8/(1-B8)*$B$1</f>
+      <c r="F8" s="1">
+        <f t="shared" si="0"/>
         <v>19.800000000000004</v>
       </c>
-      <c r="F8" s="1">
-        <f>E8-E7</f>
+      <c r="G8" s="1">
+        <f>F8-F7</f>
         <v>13.200000000000003</v>
       </c>
-      <c r="G8">
-        <f t="shared" ref="G8" si="2">B8*3.3</f>
+      <c r="H8">
+        <f t="shared" ref="H8" si="4">C8*3.3</f>
         <v>2.9699999999999998</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>28</v>
       </c>
-      <c r="K8">
-        <v>12</v>
-      </c>
-      <c r="M8" s="3">
-        <f>$C$12*(K8+K7+K6+K5+K4+K3)/($B$1+K8+K7+K6+K5+K4+K3)</f>
-        <v>2.9504573904670197</v>
+      <c r="L8">
+        <v>13</v>
       </c>
       <c r="N8" s="3">
-        <f t="shared" si="1"/>
-        <v>0.47827951133361113</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+        <f>$D$12*(L8+L7+L6+L5+L4+L3)/($C$1+L8+L7+L6+L5+L4+L3)</f>
+        <v>2.9693989071038249</v>
+      </c>
+      <c r="O8" s="3">
+        <f t="shared" si="3"/>
+        <v>0.47966676424668186</v>
+      </c>
+      <c r="Q8" s="4">
+        <f t="shared" si="2"/>
+        <v>3685.6539162112931</v>
+      </c>
+      <c r="S8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>3.3</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>30</v>
       </c>
-      <c r="M9" s="3">
+      <c r="N9" s="3">
         <v>3.3</v>
       </c>
-      <c r="N9" s="3">
-        <f t="shared" si="1"/>
-        <v>0.34954260953298011</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B12" t="s">
+      <c r="O9" s="3">
+        <f t="shared" si="3"/>
+        <v>0.3306010928961749</v>
+      </c>
+      <c r="Q9" s="4">
+        <f t="shared" si="2"/>
+        <v>4096</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="C12" t="s">
         <v>11</v>
       </c>
-      <c r="C12">
+      <c r="D12">
         <v>3.3</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B13" t="s">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="C13" t="s">
         <v>12</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Alle Hardware Änderungen commited.  Cae ist jetzt bezüglich der Ausbrüche für Knöpfe etwas vergrößert worde und die PAssung für den Drehknopf wurde etwas enger gemacht für besseren Halt
</commit_message>
<xml_diff>
--- a/hardware/DuploTrainController NG/5 Buttons an ADC.xlsx
+++ b/hardware/DuploTrainController NG/5 Buttons an ADC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/SSD1000/2_Workbench/2_HW_Projekte/4_Realisierte_Projekte/20_Duplo Train Controller NG/DuploTrain-NG/hardware/DuploTrainController NG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78900CBA-AB6F-514C-8BB2-4656FABF8632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FF687E0-54A8-1A4D-BDD3-0079CB8BEFF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30620" yWindow="1340" windowWidth="28800" windowHeight="16260" xr2:uid="{3208A821-9F98-A04C-982F-D10FE78BA69E}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
   <si>
     <t>R1</t>
   </si>
@@ -100,12 +100,6 @@
     <t>delta</t>
   </si>
   <si>
-    <t>closed</t>
-  </si>
-  <si>
-    <t>Encoder Btn</t>
-  </si>
-  <si>
     <t>Record</t>
   </si>
   <si>
@@ -124,18 +118,12 @@
     <t>Sound Cycle</t>
   </si>
   <si>
-    <t>Funktion</t>
-  </si>
-  <si>
     <t>alle offen</t>
   </si>
   <si>
     <t>R E12 in k</t>
   </si>
   <si>
-    <t>ADC Wert</t>
-  </si>
-  <si>
     <t>Sound</t>
   </si>
   <si>
@@ -143,6 +131,12 @@
   </si>
   <si>
     <t>Button</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>ADC Value</t>
   </si>
 </sst>
 </file>
@@ -188,12 +182,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -518,342 +523,453 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1">
         <v>2.2000000000000002</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F1" t="s">
+      <c r="E1" s="1"/>
+      <c r="F1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>16</v>
       </c>
+      <c r="I1" s="1"/>
       <c r="J1" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="L1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="N1" t="s">
-        <v>16</v>
-      </c>
-      <c r="O1" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>32</v>
-      </c>
-      <c r="S1" t="s">
-        <v>35</v>
-      </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1">
+        <v>0.15</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3">
-        <v>0.15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>0</v>
-      </c>
-      <c r="F3" s="1">
+      <c r="F3" s="3">
         <f t="shared" ref="F3:F8" si="0">C3/(1-C3)*$C$1</f>
         <v>0.38823529411764712</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="3">
         <f>F3</f>
         <v>0.38823529411764712</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="1">
         <f>C3*3.3</f>
         <v>0.49499999999999994</v>
       </c>
-      <c r="J3" t="s">
-        <v>23</v>
-      </c>
-      <c r="L3">
+      <c r="I3" s="1"/>
+      <c r="J3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1">
         <v>0.43</v>
       </c>
-      <c r="N3" s="3">
+      <c r="M3" s="1"/>
+      <c r="N3" s="4">
         <f>$D$12*L3/($C$1+L3)</f>
         <v>0.53954372623574132</v>
       </c>
-      <c r="O3" s="3">
+      <c r="O3" s="4">
         <f>N3</f>
         <v>0.53954372623574132</v>
       </c>
-      <c r="Q3" s="4">
+      <c r="P3" s="1"/>
+      <c r="Q3" s="5">
         <f>N3/$N$9*4096</f>
         <v>669.68821292775658</v>
       </c>
-      <c r="S3" t="s">
-        <v>23</v>
+      <c r="R3" s="1"/>
+      <c r="S3" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C4">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1">
         <v>0.3</v>
       </c>
-      <c r="E4" t="s">
+      <c r="D4" s="1"/>
+      <c r="E4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="3">
         <f t="shared" si="0"/>
         <v>0.94285714285714295</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="3">
         <f>F4-G3</f>
         <v>0.55462184873949583</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="1">
         <f t="shared" ref="H4:H7" si="1">C4*3.3</f>
         <v>0.98999999999999988</v>
       </c>
-      <c r="J4" t="s">
-        <v>24</v>
-      </c>
-      <c r="L4">
+      <c r="I4" s="1"/>
+      <c r="J4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1">
         <v>0.62</v>
       </c>
-      <c r="N4" s="3">
+      <c r="M4" s="1"/>
+      <c r="N4" s="4">
         <f>$D$12*(L4+L3)/($C$1+L4+L3)</f>
         <v>1.066153846153846</v>
       </c>
-      <c r="O4" s="3">
+      <c r="O4" s="4">
         <f>N4-N3</f>
         <v>0.52661011991810469</v>
       </c>
-      <c r="Q4" s="4">
+      <c r="P4" s="1"/>
+      <c r="Q4" s="5">
         <f t="shared" ref="Q4:Q9" si="2">N4/$N$9*4096</f>
         <v>1323.3230769230768</v>
       </c>
-      <c r="S4" t="s">
-        <v>24</v>
+      <c r="R4" s="1"/>
+      <c r="S4" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C5">
+      <c r="B5" s="1"/>
+      <c r="C5" s="1">
         <v>0.45</v>
       </c>
-      <c r="E5" t="s">
+      <c r="D5" s="1"/>
+      <c r="E5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="3">
         <f t="shared" si="0"/>
         <v>1.8</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="3">
         <f>F5-F4</f>
         <v>0.8571428571428571</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="1">
         <f t="shared" si="1"/>
         <v>1.4849999999999999</v>
       </c>
-      <c r="J5" t="s">
-        <v>25</v>
-      </c>
-      <c r="L5">
+      <c r="I5" s="1"/>
+      <c r="J5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1">
         <v>0.91</v>
       </c>
-      <c r="N5" s="3">
+      <c r="M5" s="1"/>
+      <c r="N5" s="4">
         <f>$D$12*(L5+L4+L3)/($C$1+L5+L4+L3)</f>
         <v>1.5548076923076923</v>
       </c>
-      <c r="O5" s="3">
+      <c r="O5" s="4">
         <f t="shared" ref="O5:O9" si="3">N5-N4</f>
         <v>0.48865384615384633</v>
       </c>
-      <c r="Q5" s="4">
+      <c r="P5" s="1"/>
+      <c r="Q5" s="5">
         <f t="shared" si="2"/>
         <v>1929.846153846154</v>
       </c>
-      <c r="S5" t="s">
-        <v>25</v>
+      <c r="R5" s="1"/>
+      <c r="S5" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C6">
+      <c r="B6" s="1"/>
+      <c r="C6" s="1">
         <v>0.6</v>
       </c>
-      <c r="E6" t="s">
+      <c r="D6" s="1"/>
+      <c r="E6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="3">
         <f t="shared" si="0"/>
         <v>3.3</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="3">
         <f>F6-F5</f>
         <v>1.4999999999999998</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="1">
         <f t="shared" si="1"/>
         <v>1.9799999999999998</v>
       </c>
-      <c r="J6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L6">
+      <c r="I6" s="1"/>
+      <c r="J6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1">
         <v>1.5</v>
       </c>
-      <c r="N6" s="3">
+      <c r="M6" s="1"/>
+      <c r="N6" s="4">
         <f>$D$12*(L6+L5+L4+L3)/($C$1+L6+L5+L4+L3)</f>
         <v>2.0173144876325089</v>
       </c>
-      <c r="O6" s="3">
+      <c r="O6" s="4">
         <f t="shared" si="3"/>
         <v>0.46250679532481653</v>
       </c>
-      <c r="Q6" s="4">
+      <c r="P6" s="1"/>
+      <c r="Q6" s="5">
         <f t="shared" si="2"/>
         <v>2503.9151943462898</v>
       </c>
-      <c r="S6" t="s">
-        <v>26</v>
+      <c r="R6" s="1"/>
+      <c r="S6" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C7">
+      <c r="B7" s="1"/>
+      <c r="C7" s="1">
         <v>0.75</v>
       </c>
-      <c r="E7" t="s">
+      <c r="D7" s="1"/>
+      <c r="E7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7" s="3">
         <f t="shared" si="0"/>
         <v>6.6000000000000005</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G7" s="3">
         <f>F7-F6</f>
         <v>3.3000000000000007</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="1">
         <f t="shared" si="1"/>
         <v>2.4749999999999996</v>
       </c>
-      <c r="J7" t="s">
-        <v>27</v>
-      </c>
-      <c r="L7">
+      <c r="I7" s="1"/>
+      <c r="J7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1">
         <v>3.3</v>
       </c>
-      <c r="N7" s="3">
+      <c r="M7" s="1"/>
+      <c r="N7" s="4">
         <f>$D$12*(L7+L6+L5+L4+L3)/($C$1+L7+L6+L5+L4+L3)</f>
         <v>2.4897321428571431</v>
       </c>
-      <c r="O7" s="3">
+      <c r="O7" s="4">
         <f t="shared" si="3"/>
         <v>0.47241765522463419</v>
       </c>
-      <c r="Q7" s="4">
+      <c r="P7" s="1"/>
+      <c r="Q7" s="5">
         <f t="shared" si="2"/>
         <v>3090.2857142857147</v>
       </c>
-      <c r="S7" t="s">
-        <v>34</v>
+      <c r="R7" s="1"/>
+      <c r="S7" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C8">
+      <c r="B8" s="1"/>
+      <c r="C8" s="1">
         <v>0.9</v>
       </c>
-      <c r="E8" t="s">
+      <c r="D8" s="1"/>
+      <c r="E8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="3">
         <f t="shared" si="0"/>
         <v>19.800000000000004</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8" s="3">
         <f>F8-F7</f>
         <v>13.200000000000003</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="1">
         <f t="shared" ref="H8" si="4">C8*3.3</f>
         <v>2.9699999999999998</v>
       </c>
-      <c r="J8" t="s">
-        <v>28</v>
-      </c>
-      <c r="L8">
+      <c r="I8" s="1"/>
+      <c r="J8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1">
         <v>13</v>
       </c>
-      <c r="N8" s="3">
+      <c r="M8" s="1"/>
+      <c r="N8" s="4">
         <f>$D$12*(L8+L7+L6+L5+L4+L3)/($C$1+L8+L7+L6+L5+L4+L3)</f>
         <v>2.9693989071038249</v>
       </c>
-      <c r="O8" s="3">
+      <c r="O8" s="4">
         <f t="shared" si="3"/>
         <v>0.47966676424668186</v>
       </c>
-      <c r="Q8" s="4">
+      <c r="P8" s="1"/>
+      <c r="Q8" s="5">
         <f t="shared" si="2"/>
         <v>3685.6539162112931</v>
       </c>
-      <c r="S8" t="s">
-        <v>33</v>
+      <c r="R8" s="1"/>
+      <c r="S8" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="H9">
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1">
         <v>3.3</v>
       </c>
-      <c r="J9" t="s">
-        <v>30</v>
-      </c>
-      <c r="N9" s="3">
+      <c r="I9" s="1"/>
+      <c r="J9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="4">
         <v>3.3</v>
       </c>
-      <c r="O9" s="3">
+      <c r="O9" s="4">
         <f t="shared" si="3"/>
         <v>0.3306010928961749</v>
       </c>
-      <c r="Q9" s="4">
+      <c r="P9" s="1"/>
+      <c r="Q9" s="5">
         <f t="shared" si="2"/>
         <v>4096</v>
       </c>
+      <c r="R9" s="1"/>
+      <c r="S9" s="1"/>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="1"/>
+      <c r="R10" s="1"/>
+      <c r="S10" s="1"/>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="1"/>
+      <c r="R11" s="1"/>
+      <c r="S11" s="1"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="C12" t="s">

</xml_diff>